<commit_message>
Add sales model tabs to CRM review workbook
Extends the workbook with the agreed CRM sales model: the four-layer
object model (Club, Lead, Task, Opportunity) with build status, the Lead
lane and its manual conversion, the Task lane with all three sources
(inbound trial request, trial-expiry scan, renewal scan) and dedupe
keys, the Opportunity pipeline and bundle/ARR rules, and the two-way
flow with the team's daily views.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmQtZyzk2RanBLBqCtiCpM
</commit_message>
<xml_diff>
--- a/BetterCricket-CRM-telemetry-and-fields.xlsx
+++ b/BetterCricket-CRM-telemetry-and-fields.xlsx
@@ -14,6 +14,11 @@
     <sheet name="4. Refresh paths" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="5. Write-back (Twenty to BC)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="6. Gaps to review" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="7. Sales model" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="8. Lead lane" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="9. Task lane" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10. Opportunity pipeline" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11. Flow and views" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +73,19 @@
       <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00222222"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +117,16 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2DCDB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -128,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -156,6 +182,21 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -537,6 +578,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -605,13 +647,850 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>1 Telemetry sources | 2 Company field logic | 3 Engagement score | 4 Refresh paths | 5 Write-back (Twenty to BC) | 6 Gaps to review</t>
+          <t>1 Telemetry | 2 Company field logic | 3 Engagement score | 4 Refresh paths | 5 Write-back | 6 Gaps | 7 Sales model | 8 Lead lane | 9 Task lane | 10 Opportunity pipeline | 11 Flow &amp; views</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 9 — Task lane (must-do, must-confirm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Actions a human must carry out and confirm. All sources flow through the module_action_requests queue and mirror to a native Twenty Task, so nothing is lost. Dedupe keys stop a daily scan re-raising the same task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Trigger condition</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Task raised</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Dedupe external_ref</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>The three task sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Inbound trial request (new club)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>trial requested AND club not a customer AND no BetterStats trial started</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Initiate sync + start BetterStats trial for {club}</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>req:{club}:{module}</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>a few days</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Inbound trial request (existing club)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>trial requested AND club already synced / customer</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Enable {module} trial for {club}</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>req:{club}:{module}</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>a few days</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Trial expiry scan (daily 07:00)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>OrgModuleSubscription status=trial AND trial_ends_at within 7 days</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Trial ending {date}: {module} for {club}, follow up to convert</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>trial_end:{sub_id}:{trial_ends_at}</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>before trial end</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Renewal scan (daily 07:00)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>paid subscription AND renewal_date within 30 days (org.renewal_date fallback)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Renewal due {date}: {module} for {club}, confirm renewal</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>renewal:{sub_id}:{renewal_date}</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>before renewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Mechanics</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>module_action_requests (status outstanding to done) is the single queue; each outstanding row mirrors to a Twenty Task</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="15" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>back-office default, or the club owner if set (config item)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="14" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>staff mark the request done and the Task closes; the sync itself runs in BetterCricket (nothing auto-provisions)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Auto-close</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>trial converts to paid, or renewal_date rolls forward: the next scan closes the stale Task</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Visibility</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Action queue view (open Tasks by due date) + the Club timeline</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>trials 7 days, renewals 30 days, both tunable; optional second renewal nudge at 7 days</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="14" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 10 — Opportunity (the deal board)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Created only by converting a Lead. Club-centric with per-module attention and a bundle option. The board shows only clubs someone has chosen to pursue, which keeps it concise for a small team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Notes / decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>one acquisition Deal per club at a time</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>expansion later = a new Cross-sell deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Stages</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Qualifying / Demo or Trial / Proposal / Committee / Won / Lost</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>account states (Target/Contacted/Engaged) stay on the Club, not the deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>modulesInScope</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Core always + any add-ons in play</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>field exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>salesMotion</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>New Sale / Cross-sell / Renewal</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>new field</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>bundleApplies</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>true only on the first subscription</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>derivable from 'club has no active sub yet'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>amount (ARR)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>bundle price on acquisition; standard + optional discretionary discount on expansion</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>current _arr always applies the bundle discount by module count: correct for acquisition, over-discounts expansion (decide)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>oppSource</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>inbound form / outbound campaign / referral / directory</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>field exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>lostReason</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>not interested / no budget / competitor / no response / other</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>field exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>bcOpportunityKey</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>club + motion</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>idempotency key, field exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>nextStep / nextFollowUpDate</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>free text + date</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>new fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Won</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>BetterCricket provisions the subscription</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>via opportunity.updated webhook</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 11 — Two-way flow and the daily views</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>What moves each way and when, then the saved views the two-person team works from. Keeping the three queues separate stops 'must do' getting buried under 'might chase'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>What moves</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Trigger / cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>BetterCricket to CRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BC to CRM</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>identity, module/subscription state, engagement rollup, suppression flags, directory arrays</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Export (manual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>BC to CRM</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>engagement rollup (score, tier, sessions, last-seen)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Daily 06:00 + on-demand button</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>BC to CRM</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>modules, subscription, ARR, renewal, billing</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Module-change hook (near real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>BC to CRM</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Telemetry events</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>BC to CRM</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Request queue + daily 07:00 trial/renewal scan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>BC to CRM</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Person suppression, contactSource, lastCampaign</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>SES + Contact Us (real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>CRM to BetterCricket</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>CRM to BC</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Lead conversion creates an Opportunity</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>lead.updated webhook / Workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>CRM to BC</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Opportunity Won provisions the club</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>opportunity.updated webhook</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>CRM to BC</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Task done closes its request</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>task webhook (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>CRM to BC</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>module flagged interested raises a request</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>company.updated webhook (exists)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>The daily views</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Action queue</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>open Tasks by due date</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>the must-clear list</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Lead inbox</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>New + Working Leads</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>triage</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Opportunity board</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>pipeline kanban</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>deals to close</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Club / Contact lists</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>filter and segment</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>build the next campaign</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2717,4 +3596,581 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 7 — CRM object model (agreed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>The four working layers after simplification. Detailed telemetry stays in BetterCricket; the CRM holds the account, the interest queue, the action queue and the deal board. Status colours: green exists, amber scaffolded/partial, orange new, red remove.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Key fields</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Created by</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Build status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Club (Company)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>The account: every targeted club</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>lifecycle stage; module status (paid/trial/interested); engagement rollup; Association array (read-only, from directory); optional Primary Association; ARR; renewal; billing</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Directory export</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Partly exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Contact (Person)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>A club officer</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>identity; single home club; Club array (read-only, every club served); role; subscribed/bounced; contactSource; lastCampaign</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Directory export</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Partly exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Lead (custom)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Passive interest triage queue</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>link to Club; source; signal summary; engagement tier; modulesOfInterest; status (New/Working/Converted/Discarded); 'Modules to pursue' multi-select (convert trigger)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Auto, from telemetry</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Task (native)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Must-do action, confirmed</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>linked Club; title; body; assignee; due date; status To-do/Done</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Auto, from a request</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Opportunity (Deal)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Active deal to Won or Lost</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>modulesInScope; salesMotion; bundleApplies; amount (ARR); stage; oppSource; lostReason; bcOpportunityKey; nextStep; nextFollowUpDate</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Manual, Lead conversion</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Scaffolded</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Removed / simplified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Memberships (clubAssociation)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Club-to-association junction</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Replaced by the Club Association array</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Officer roles (personClub)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Contact-to-club junction</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Replaced by the Contact Club array</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Association (object)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Association as a record</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Replaced by the read-only arrays on Club</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Touchpoint / Email (objects)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Per-event / per-campaign records</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Left empty. Detailed email + web telemetry stays in BetterCricket / BetterComms</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 8 — Lead lane (telemetry to interest, then manual convert)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Telemetry raises Leads, not Opportunities. A Lead is a passive triage item; converting it is a deliberate human step. One Lead per club, refreshed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Triggers that raise / refresh a Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Club responds or engages meaningfully</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>reply, call booked, a click plus a question</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Contact Us enquiry</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>POST /public/contact naming interest</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>requested_trial_modules gains a module</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>also raises a Task, see Sheet 9</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Trial started</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>also raises a Task, see Sheet 9</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Engagement crosses Hot</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>raise as a suggested Lead for a human to accept</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Lead fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>New / Working / Converted / Discarded</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>outbound campaign / website / email engagement / contact us</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>modulesOfInterest</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>from requested_trial_modules</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Modules to pursue (multi-select)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>the convert trigger; also carries the deal scope</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Conversion to an Opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Convert action</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>user sets 'Modules to pursue' from empty to non-empty</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Effect</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>create Opportunity, copy those modules into modulesInScope, set Lead = Converted</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>No duplicates</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>keyed on bcOpportunityKey (club + motion); later edits update the same deal</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Mechanism</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>our webhook handler on lead.updated (recommended) OR a native Twenty Workflow (version-sensitive)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>status = Discarded, optional write-back to not_interested in BetterCricket</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add go-live seed section to Lead and Task lanes
Documents the one-time initialisation that both event-driven lanes need
at cutover: a Leads backfill over the exported subset (qualifying signals
only, keyed lead:{club}), a mirror of open module_action_requests to
Twenty Tasks, and a note that the daily trial/renewal scan self-seeds on
its first run. All idempotent via the same keys the live triggers use.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmQtZyzk2RanBLBqCtiCpM
</commit_message>
<xml_diff>
--- a/BetterCricket-CRM-telemetry-and-fields.xlsx
+++ b/BetterCricket-CRM-telemetry-and-fields.xlsx
@@ -128,7 +128,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -150,11 +150,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -199,6 +243,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -578,7 +624,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -665,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -722,6 +767,10 @@
           <t>The three task sources</t>
         </is>
       </c>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -837,6 +886,10 @@
           <t>Mechanics</t>
         </is>
       </c>
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -928,11 +981,88 @@
       <c r="D15" s="14" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Go-live seed (one-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Outstanding requests mirror</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>each open module_action_requests row becomes a Twenty Task</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>run once at go-live</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>(reuses each request external_ref)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>per due</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Trials / renewals self-seed</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>no backfill needed: the first 07:00 scan is a scan over current dates, so it raises every in-window trial expiry and renewal on its first run</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>just run the scan once after go-live</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>trial_end / renewal refs</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>the seed reuses the same external_ref keys as the live triggers, so seed + events never duplicate</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="14" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A4:E4"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1231,6 +1361,8 @@
           <t>BetterCricket to CRM</t>
         </is>
       </c>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1340,6 +1472,8 @@
           <t>CRM to BetterCricket</t>
         </is>
       </c>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1415,6 +1549,8 @@
           <t>The daily views</t>
         </is>
       </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -3796,6 +3932,10 @@
           <t>Removed / simplified</t>
         </is>
       </c>
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -3921,7 +4061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3966,6 +4106,8 @@
           <t>Triggers that raise / refresh a Lead</t>
         </is>
       </c>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -4038,6 +4180,8 @@
           <t>Lead fields</t>
         </is>
       </c>
+      <c r="B10" s="16" t="n"/>
+      <c r="C10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -4097,6 +4241,8 @@
           <t>Conversion to an Opportunity</t>
         </is>
       </c>
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -4163,10 +4309,70 @@
       </c>
       <c r="C20" s="9" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Go-live seed (one-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Leads backfill</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>walk every exported club (twenty_links) and create a Lead for each that qualifies now: requested_trial_modules set, demo_status = in_trial, or inSalesCycle true (already computed by the engagement rollup)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Selector rule</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>qualifying signals only, never 'has been emailed', so Contacted-only clubs get no Lead (same rule that keeps the board clean day to day)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Fields</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>source + modulesOfInterest from the strongest current signal; status New, or Working if a trial is already live</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>keyed lead:{club} so a re-run, or a live event firing right after, never doubles up</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>

</xml_diff>